<commit_message>
first draft of explorer and includer
</commit_message>
<xml_diff>
--- a/input_data/sna_country_data/URY/cei.xlsx
+++ b/input_data/sna_country_data/URY/cei.xlsx
@@ -11,13 +11,15 @@
     <sheet name="2017" sheetId="3" r:id="rId5"/>
     <sheet name="2018" sheetId="4" r:id="rId6"/>
     <sheet name="2019" sheetId="5" r:id="rId7"/>
+    <sheet name="2020" sheetId="6" r:id="rId8"/>
+    <sheet name="2021" sheetId="7" r:id="rId9"/>
   </sheets>
   <calcPr calcId="125725" fullCalcOnLoad="true"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9840" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10414" uniqueCount="76">
   <si>
     <t>code</t>
   </si>
@@ -863,10 +865,10 @@
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1">
+        <v>-3264.8749993161441</v>
+      </c>
+      <c r="F27" s="1">
         <v>-3264.8749993161591</v>
-      </c>
-      <c r="F27" s="1">
-        <v>-3264.8749993161441</v>
       </c>
       <c r="G27" s="1">
         <v>65128.014697722727</v>
@@ -943,10 +945,10 @@
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1">
+        <v>-3264.8749993161591</v>
+      </c>
+      <c r="F31" s="1">
         <v>-3264.8749993161441</v>
-      </c>
-      <c r="F31" s="1">
-        <v>-3264.8749993161591</v>
       </c>
       <c r="G31" s="1">
         <v>65128.014697722727</v>
@@ -1017,10 +1019,10 @@
         <v>-25147.551874929632</v>
       </c>
       <c r="G34" s="1">
-        <v>25446.753598644718</v>
+        <v>25446.753598644849</v>
       </c>
       <c r="H34" s="1">
-        <v>25446.753598644718</v>
+        <v>25446.753598644849</v>
       </c>
     </row>
     <row r="35">
@@ -1043,63 +1045,63 @@
         <v>-25147.551874929632</v>
       </c>
       <c r="G35" s="1">
-        <v>25446.753598644849</v>
+        <v>25446.753598644718</v>
       </c>
       <c r="H35" s="1">
-        <v>25446.753598644849</v>
+        <v>25446.753598644718</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B36" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>926.5806651800001</v>
-      </c>
-      <c r="F36" s="1"/>
+        <v>79482.446760280014</v>
+      </c>
+      <c r="F36" s="1">
+        <v>79482.446760280014</v>
+      </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B37" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>79482.446760280014</v>
-      </c>
-      <c r="F37" s="1">
-        <v>79482.446760280014</v>
-      </c>
+        <v>113976.0975413</v>
+      </c>
+      <c r="F37" s="1"/>
       <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
+      <c r="H37" s="1">
+        <v>137582.86030768359</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>113976.0975413</v>
+        <v>926.5806651800001</v>
       </c>
       <c r="F38" s="1"/>
       <c r="G38" s="1"/>
-      <c r="H38" s="1">
-        <v>137582.86030768359</v>
-      </c>
+      <c r="H38" s="1"/>
     </row>
   </sheetData>
 </worksheet>
@@ -1685,7 +1687,7 @@
         <v>-10570.43407502865</v>
       </c>
       <c r="F27" s="1">
-        <v>-10570.434075028639</v>
+        <v>-10570.43407502865</v>
       </c>
       <c r="G27" s="1">
         <v>124508.5573505638</v>
@@ -1765,7 +1767,7 @@
         <v>-10570.434075028639</v>
       </c>
       <c r="F31" s="1">
-        <v>-10570.43407502865</v>
+        <v>-10570.434075028639</v>
       </c>
       <c r="G31" s="1">
         <v>124508.5573505638</v>
@@ -1829,7 +1831,7 @@
         <v>-14574.43484844782</v>
       </c>
       <c r="D34" s="1">
-        <v>-14574.43484844782</v>
+        <v>-14574.434848447811</v>
       </c>
       <c r="E34" s="1">
         <v>-66950.582658753847</v>
@@ -1838,10 +1840,10 @@
         <v>-66950.582658753861</v>
       </c>
       <c r="G34" s="1">
-        <v>55330.055140544697</v>
+        <v>55330.055140544151</v>
       </c>
       <c r="H34" s="1">
-        <v>55330.055140544697</v>
+        <v>55330.055140544151</v>
       </c>
     </row>
     <row r="35">
@@ -1855,7 +1857,7 @@
         <v>-14574.434848447811</v>
       </c>
       <c r="D35" s="1">
-        <v>-14574.434848447811</v>
+        <v>-14574.43484844782</v>
       </c>
       <c r="E35" s="1">
         <v>-66950.582658753861</v>
@@ -1864,63 +1866,63 @@
         <v>-66950.582658753847</v>
       </c>
       <c r="G35" s="1">
-        <v>55330.055140544151</v>
+        <v>55330.055140544697</v>
       </c>
       <c r="H35" s="1">
-        <v>55330.055140544151</v>
+        <v>55330.055140544697</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>147042.35994689999</v>
-      </c>
-      <c r="F36" s="1">
-        <v>147042.21094677999</v>
-      </c>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
+        <v>181558.9914336357</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1">
+        <v>310.92989817709997</v>
+      </c>
+      <c r="H36" s="1">
+        <v>223683.25268700649</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B37" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>181558.9914336357</v>
+        <v>1410.7265588499999</v>
       </c>
       <c r="F37" s="1"/>
-      <c r="G37" s="1">
-        <v>310.92989817709997</v>
-      </c>
-      <c r="H37" s="1">
-        <v>223683.25268700649</v>
-      </c>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B38" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>1410.7265588499999</v>
-      </c>
-      <c r="F38" s="1"/>
+        <v>147042.35994689999</v>
+      </c>
+      <c r="F38" s="1">
+        <v>147042.21094677999</v>
+      </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
@@ -2507,7 +2509,7 @@
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1">
-        <v>-25017.388782343201</v>
+        <v>-25017.38878234318</v>
       </c>
       <c r="F27" s="1">
         <v>-25017.388782343201</v>
@@ -2587,7 +2589,7 @@
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1">
-        <v>-25017.38878234318</v>
+        <v>-25017.388782343201</v>
       </c>
       <c r="F31" s="1">
         <v>-25017.38878234318</v>
@@ -2654,10 +2656,10 @@
         <v>-4009.0753441289771</v>
       </c>
       <c r="D34" s="1">
-        <v>-4009.0753441289771</v>
+        <v>-4009.0753441289712</v>
       </c>
       <c r="E34" s="1">
-        <v>-63565.770979082881</v>
+        <v>-63565.818181042087</v>
       </c>
       <c r="F34" s="1">
         <v>-63565.770979082881</v>
@@ -2680,10 +2682,10 @@
         <v>-4009.0753441289712</v>
       </c>
       <c r="D35" s="1">
-        <v>-4009.0753441289712</v>
+        <v>-4009.0753441289771</v>
       </c>
       <c r="E35" s="1">
-        <v>-63565.818181042087</v>
+        <v>-63565.770979082881</v>
       </c>
       <c r="F35" s="1">
         <v>-63565.818181042087</v>
@@ -2697,55 +2699,55 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B36" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>1378.685344355712</v>
+        <v>201604.21968480741</v>
       </c>
       <c r="F36" s="1"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
+      <c r="G36" s="1">
+        <v>337.34758922499998</v>
+      </c>
+      <c r="H36" s="1">
+        <v>253381.7166756459</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B37" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>201604.21968480741</v>
-      </c>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1">
-        <v>337.34758922499998</v>
-      </c>
-      <c r="H37" s="1">
-        <v>253381.7166756459</v>
-      </c>
+        <v>170013.75605207999</v>
+      </c>
+      <c r="F37" s="1">
+        <v>170013.75605207999</v>
+      </c>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>170013.75605207999</v>
-      </c>
-      <c r="F38" s="1">
-        <v>170013.75605207999</v>
-      </c>
+        <v>1378.685344355712</v>
+      </c>
+      <c r="F38" s="1"/>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
     </row>
@@ -3479,13 +3481,13 @@
         <v>-49773.892247342999</v>
       </c>
       <c r="F34" s="1">
-        <v>-49773.892247342999</v>
+        <v>-49773.892247343349</v>
       </c>
       <c r="G34" s="1">
         <v>33283.712597372418</v>
       </c>
       <c r="H34" s="1">
-        <v>33283.712597372418</v>
+        <v>33283.712597372112</v>
       </c>
     </row>
     <row r="35">
@@ -3505,13 +3507,13 @@
         <v>-49773.892247343349</v>
       </c>
       <c r="F35" s="1">
-        <v>-49773.892247343349</v>
+        <v>-49773.892247342999</v>
       </c>
       <c r="G35" s="1">
         <v>33283.712597372112</v>
       </c>
       <c r="H35" s="1">
-        <v>33283.712597372112</v>
+        <v>33283.712597372418</v>
       </c>
     </row>
     <row r="36">
@@ -4149,10 +4151,10 @@
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1">
+        <v>-47487.012322160823</v>
+      </c>
+      <c r="F27" s="1">
         <v>-47487.012322160852</v>
-      </c>
-      <c r="F27" s="1">
-        <v>-47487.012322160823</v>
       </c>
       <c r="G27" s="1">
         <v>137422.3722114753</v>
@@ -4227,10 +4229,10 @@
       <c r="C31" s="1"/>
       <c r="D31" s="1"/>
       <c r="E31" s="1">
+        <v>-47487.012322160852</v>
+      </c>
+      <c r="F31" s="1">
         <v>-47487.012322160823</v>
-      </c>
-      <c r="F31" s="1">
-        <v>-47487.012322160852</v>
       </c>
       <c r="G31" s="1">
         <v>137422.3722114753</v>
@@ -4300,10 +4302,10 @@
         <v>-63947.039175030113</v>
       </c>
       <c r="F34" s="1">
-        <v>-63947.039175030113</v>
+        <v>-63947.039175029808</v>
       </c>
       <c r="G34" s="1">
-        <v>39248.472782472993</v>
+        <v>39248.472782472847</v>
       </c>
       <c r="H34" s="1">
         <v>39248.472782472847</v>
@@ -4326,13 +4328,1649 @@
         <v>-63947.039175029808</v>
       </c>
       <c r="F35" s="1">
-        <v>-63947.039175029808</v>
+        <v>-63947.039175030113</v>
       </c>
       <c r="G35" s="1">
-        <v>39248.472782472847</v>
+        <v>39248.472782472993</v>
       </c>
       <c r="H35" s="1">
         <v>39248.472782472993</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36" t="s">
+        <v>66</v>
+      </c>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1">
+        <v>239376.743428952</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1">
+        <v>402.67289956090139</v>
+      </c>
+      <c r="H36" s="1">
+        <v>298520.24294644757</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>33</v>
+      </c>
+      <c r="B37" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1">
+        <v>200663.39336498949</v>
+      </c>
+      <c r="F37" s="1">
+        <v>200663.39336498949</v>
+      </c>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1">
+        <v>1691.532447066628</v>
+      </c>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H38"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="1">
+        <v>-104514.67406784389</v>
+      </c>
+      <c r="D2" s="1">
+        <v>-104514.67406784389</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1">
+        <v>248943.64208872389</v>
+      </c>
+      <c r="F3" s="1">
+        <v>248943.64208872389</v>
+      </c>
+      <c r="G3" s="1">
+        <v>470818.5045513846</v>
+      </c>
+      <c r="H3" s="1">
+        <v>470818.5045513846</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1">
+        <v>290515.63883653207</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1589.3641487719749</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1">
+        <v>16917.042990926879</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1">
+        <v>255855.03423551831</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1">
+        <v>34660.604601013787</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1589.3641487719749</v>
+      </c>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1">
+        <v>16917.042990926879</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1">
+        <v>-20094.858684111801</v>
+      </c>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1">
+        <v>-3424.6937240000002</v>
+      </c>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1">
+        <v>-16670.164960111801</v>
+      </c>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1">
+        <v>186501.3272761718</v>
+      </c>
+      <c r="H10" s="1">
+        <v>186501.3272761718</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1">
+        <v>744.17415905056737</v>
+      </c>
+      <c r="F11" s="1">
+        <v>744.17415905056737</v>
+      </c>
+      <c r="G11" s="1">
+        <v>208793.31727426461</v>
+      </c>
+      <c r="H11" s="1">
+        <v>208793.31727426461</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="1">
+        <v>-149.5741136579793</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1">
+        <v>246610.10378090141</v>
+      </c>
+      <c r="G12" s="1">
+        <v>964516.23533725785</v>
+      </c>
+      <c r="H12" s="1">
+        <v>58606.817010021281</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="1">
+        <v>151856.17438438139</v>
+      </c>
+      <c r="D13" s="1">
+        <v>30555.43229442582</v>
+      </c>
+      <c r="E13" s="1">
+        <v>79370.097059280903</v>
+      </c>
+      <c r="F13" s="1">
+        <v>68905.215310340413</v>
+      </c>
+      <c r="G13" s="1">
+        <v>196071.41583780959</v>
+      </c>
+      <c r="H13" s="1">
+        <v>24681.605703741461</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="1">
+        <v>54754.723496312057</v>
+      </c>
+      <c r="D14" s="1">
+        <v>33544.679116953143</v>
+      </c>
+      <c r="E14" s="1">
+        <v>11018.02669235646</v>
+      </c>
+      <c r="F14" s="1">
+        <v>68905.215310340413</v>
+      </c>
+      <c r="G14" s="1">
+        <v>18312.725199786091</v>
+      </c>
+      <c r="H14" s="1">
+        <v>24681.605703741461</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="1">
+        <v>97101.450888069332</v>
+      </c>
+      <c r="D15" s="1">
+        <v>-2989.2468225273192</v>
+      </c>
+      <c r="E15" s="1">
+        <v>68352.070366924439</v>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1">
+        <v>177758.69063802349</v>
+      </c>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="1">
+        <v>121151.1679762976</v>
+      </c>
+      <c r="D16" s="1">
+        <v>121151.1679762976</v>
+      </c>
+      <c r="E16" s="1">
+        <v>281629.83606041141</v>
+      </c>
+      <c r="F16" s="1">
+        <v>281629.83606041141</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1531200.6900217619</v>
+      </c>
+      <c r="H16" s="1">
+        <v>1531200.6900217619</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="1">
+        <v>829.94672213900139</v>
+      </c>
+      <c r="D17" s="1">
+        <v>6471.0488226466759</v>
+      </c>
+      <c r="E17" s="1">
+        <v>177143.6583732735</v>
+      </c>
+      <c r="F17" s="1">
+        <v>53.220586556000001</v>
+      </c>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1">
+        <v>103439.93424494661</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1851.55709250523</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1">
+        <v>250754.8245620098</v>
+      </c>
+      <c r="F18" s="1">
+        <v>354136.98076916719</v>
+      </c>
+      <c r="G18" s="1">
+        <v>371603.72775322967</v>
+      </c>
+      <c r="H18" s="1">
+        <v>313623.89550054661</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" s="1">
+        <v>1851.55709250523</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1">
+        <v>354136.98076916719</v>
+      </c>
+      <c r="G19" s="1">
+        <v>371161.41966917628</v>
+      </c>
+      <c r="H19" s="1">
+        <v>442.30808405340002</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="1">
+        <v>13110.58352570426</v>
+      </c>
+      <c r="D20" s="1">
+        <v>12660.168619784579</v>
+      </c>
+      <c r="E20" s="1">
+        <v>261006.27914480091</v>
+      </c>
+      <c r="F20" s="1">
+        <v>261258.07254784679</v>
+      </c>
+      <c r="G20" s="1">
+        <v>47158.262679367523</v>
+      </c>
+      <c r="H20" s="1">
+        <v>48339.543750886784</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="1">
+        <v>1.421961</v>
+      </c>
+      <c r="D21" s="1">
+        <v>2008.0292188799999</v>
+      </c>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1">
+        <v>602.00508799464785</v>
+      </c>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1">
+        <v>6521.2483581013976</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="1">
+        <v>2008.0292188799999</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1">
+        <v>848.91206396320899</v>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1">
+        <v>8013.8274215867395</v>
+      </c>
+      <c r="H22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="1">
+        <v>728.95224428820325</v>
+      </c>
+      <c r="D23" s="1">
+        <v>88.157780000000002</v>
+      </c>
+      <c r="E23" s="1">
+        <v>88.157780000000002</v>
+      </c>
+      <c r="F23" s="1">
+        <v>728.95224428820325</v>
+      </c>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="1">
+        <v>10372.18010153606</v>
+      </c>
+      <c r="D24" s="1">
+        <v>10563.981620904589</v>
+      </c>
+      <c r="E24" s="1">
+        <v>16195.29706350237</v>
+      </c>
+      <c r="F24" s="1">
+        <v>17678.695071503971</v>
+      </c>
+      <c r="G24" s="1">
+        <v>39144.435257780773</v>
+      </c>
+      <c r="H24" s="1">
+        <v>41818.295392785381</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="1">
+        <v>117812.0378742148</v>
+      </c>
+      <c r="D25" s="1">
+        <v>117812.0378742148</v>
+      </c>
+      <c r="E25" s="1">
+        <v>355086.32423692557</v>
+      </c>
+      <c r="F25" s="1">
+        <v>355086.32423692557</v>
+      </c>
+      <c r="G25" s="1">
+        <v>1484559.3069579799</v>
+      </c>
+      <c r="H25" s="1">
+        <v>1484559.3069579799</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1">
+        <v>43550.766861969081</v>
+      </c>
+      <c r="H26" s="1"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1">
+        <v>-43451.658659149427</v>
+      </c>
+      <c r="F27" s="1">
+        <v>-43451.658659149427</v>
+      </c>
+      <c r="G27" s="1">
+        <v>153931.3940779226</v>
+      </c>
+      <c r="H27" s="1">
+        <v>153931.3940779226</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1">
+        <v>231638.87160831151</v>
+      </c>
+      <c r="G28" s="1">
+        <v>239321.86905549711</v>
+      </c>
+      <c r="H28" s="1"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1">
+        <v>123447.4526286141</v>
+      </c>
+      <c r="F29" s="1">
+        <v>123447.4526286141</v>
+      </c>
+      <c r="G29" s="1">
+        <v>1723881.1760134769</v>
+      </c>
+      <c r="H29" s="1">
+        <v>1723881.1760134769</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1">
+        <v>43550.766861969081</v>
+      </c>
+      <c r="H30" s="1"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1">
+        <v>-43451.658659149427</v>
+      </c>
+      <c r="F31" s="1">
+        <v>-43451.658659149427</v>
+      </c>
+      <c r="G31" s="1">
+        <v>153931.3940779226</v>
+      </c>
+      <c r="H31" s="1">
+        <v>153931.3940779226</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="1">
+        <v>13297.36380637088</v>
+      </c>
+      <c r="D32" s="1">
+        <v>13297.36380637088</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" t="s">
+        <v>64</v>
+      </c>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1">
+        <v>-3163.35692644855</v>
+      </c>
+      <c r="E33" s="1">
+        <v>18090.690218</v>
+      </c>
+      <c r="F33" s="1">
+        <v>-15357.153292196481</v>
+      </c>
+      <c r="G33" s="1">
+        <v>8670.7725571964856</v>
+      </c>
+      <c r="H33" s="1">
+        <v>-14153.624163</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="1">
+        <v>10171.468589380889</v>
+      </c>
+      <c r="D34" s="1">
+        <v>10171.459058987501</v>
+      </c>
+      <c r="E34" s="1">
+        <v>-79545.106801385089</v>
+      </c>
+      <c r="F34" s="1">
+        <v>-79545.106801385089</v>
+      </c>
+      <c r="G34" s="1">
+        <v>66058.729479423899</v>
+      </c>
+      <c r="H34" s="1">
+        <v>66058.729479423899</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" s="1">
+        <v>10171.459058987501</v>
+      </c>
+      <c r="D35" s="1">
+        <v>10171.468589380889</v>
+      </c>
+      <c r="E35" s="1">
+        <v>-79545.106801385089</v>
+      </c>
+      <c r="F35" s="1">
+        <v>-79545.106801385089</v>
+      </c>
+      <c r="G35" s="1">
+        <v>66059.10105946564</v>
+      </c>
+      <c r="H35" s="1">
+        <v>66059.10105946564</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36" t="s">
+        <v>66</v>
+      </c>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1">
+        <v>250754.8245620098</v>
+      </c>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1">
+        <v>442.30808405340002</v>
+      </c>
+      <c r="H36" s="1">
+        <v>313181.58741649322</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>33</v>
+      </c>
+      <c r="B37" t="s">
+        <v>67</v>
+      </c>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1">
+        <v>242248.42014405999</v>
+      </c>
+      <c r="F37" s="1">
+        <v>242248.42014405999</v>
+      </c>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B38" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1">
+        <v>1625.492093275358</v>
+      </c>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:H38"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" t="s">
+        <v>73</v>
+      </c>
+      <c r="H1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="1">
+        <v>-200371.3593658637</v>
+      </c>
+      <c r="D2" s="1">
+        <v>-200371.3593658637</v>
+      </c>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1">
+        <v>264191.99060634093</v>
+      </c>
+      <c r="F3" s="1">
+        <v>264191.99060634093</v>
+      </c>
+      <c r="G3" s="1">
+        <v>501754.2312573535</v>
+      </c>
+      <c r="H3" s="1">
+        <v>501754.2312573535</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1">
+        <v>336400.38718717668</v>
+      </c>
+      <c r="F4" s="1">
+        <v>1662.9687562544871</v>
+      </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1">
+        <v>18516.856554910399</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1">
+        <v>298692.07167320402</v>
+      </c>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1">
+        <v>37708.31551397279</v>
+      </c>
+      <c r="F6" s="1">
+        <v>1662.9687562544871</v>
+      </c>
+      <c r="G6" s="1"/>
+      <c r="H6" s="1">
+        <v>18516.856554910399</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1">
+        <v>-21256.196209999998</v>
+      </c>
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="1"/>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1">
+        <v>-3607.1962100000001</v>
+      </c>
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1"/>
+      <c r="F9" s="1">
+        <v>-17649</v>
+      </c>
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1">
+        <v>198016.23387617839</v>
+      </c>
+      <c r="H10" s="1">
+        <v>198016.23387617839</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1">
+        <v>864.630246243599</v>
+      </c>
+      <c r="F11" s="1">
+        <v>864.630246243599</v>
+      </c>
+      <c r="G11" s="1">
+        <v>222382.5264923693</v>
+      </c>
+      <c r="H11" s="1">
+        <v>222382.5264923693</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="1">
+        <v>-155.06439238415939</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1">
+        <v>261664.39160384281</v>
+      </c>
+      <c r="G12" s="1">
+        <v>1051958.579323407</v>
+      </c>
+      <c r="H12" s="1">
+        <v>62838.614333895377</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" s="1">
+        <v>314231.27904663578</v>
+      </c>
+      <c r="D13" s="1">
+        <v>48491.039627563499</v>
+      </c>
+      <c r="E13" s="1">
+        <v>77992.283715817306</v>
+      </c>
+      <c r="F13" s="1">
+        <v>72672.959190910158</v>
+      </c>
+      <c r="G13" s="1">
+        <v>228007.94010357111</v>
+      </c>
+      <c r="H13" s="1">
+        <v>24065.71765295729</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="1">
+        <v>51456.424245716291</v>
+      </c>
+      <c r="D14" s="1">
+        <v>25720.518587558981</v>
+      </c>
+      <c r="E14" s="1">
+        <v>12240.36810384845</v>
+      </c>
+      <c r="F14" s="1">
+        <v>72672.959190910158</v>
+      </c>
+      <c r="G14" s="1">
+        <v>18222.007736500102</v>
+      </c>
+      <c r="H14" s="1">
+        <v>24065.71765295729</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="1">
+        <v>262774.85480091948</v>
+      </c>
+      <c r="D15" s="1">
+        <v>22770.521040004522</v>
+      </c>
+      <c r="E15" s="1">
+        <v>65751.915611968856</v>
+      </c>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1">
+        <v>209785.93236707099</v>
+      </c>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="1">
+        <v>265585.17502668808</v>
+      </c>
+      <c r="D16" s="1">
+        <v>265585.17502668808</v>
+      </c>
+      <c r="E16" s="1">
+        <v>321328.14574832749</v>
+      </c>
+      <c r="F16" s="1">
+        <v>321328.14574832749</v>
+      </c>
+      <c r="G16" s="1">
+        <v>1676299.5621425679</v>
+      </c>
+      <c r="H16" s="1">
+        <v>1676299.5621425679</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C17" s="1">
+        <v>1300.758691809164</v>
+      </c>
+      <c r="D17" s="1">
+        <v>8464.0095581612786</v>
+      </c>
+      <c r="E17" s="1">
+        <v>197849.96173044899</v>
+      </c>
+      <c r="F17" s="1">
+        <v>17.659803556</v>
+      </c>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1">
+        <v>112319.3970110997</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="1">
+        <v>2035.2769079008131</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1">
+        <v>272538.25067318691</v>
+      </c>
+      <c r="F18" s="1">
+        <v>378244.16283277201</v>
+      </c>
+      <c r="G18" s="1">
+        <v>399176.57784388593</v>
+      </c>
+      <c r="H18" s="1">
+        <v>336198.25983588898</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>51</v>
+      </c>
+      <c r="C19" s="1">
+        <v>2035.2769079008131</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1">
+        <v>378244.16283277201</v>
+      </c>
+      <c r="G19" s="1">
+        <v>398720.17342767422</v>
+      </c>
+      <c r="H19" s="1">
+        <v>456.40441621169998</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C20" s="1">
+        <v>13142.94333128056</v>
+      </c>
+      <c r="D20" s="1">
+        <v>11223.393284713609</v>
+      </c>
+      <c r="E20" s="1">
+        <v>285633.72307077801</v>
+      </c>
+      <c r="F20" s="1">
+        <v>287310.09786391503</v>
+      </c>
+      <c r="G20" s="1">
+        <v>51411.548162021252</v>
+      </c>
+      <c r="H20" s="1">
+        <v>53379.746286008769</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>57</v>
+      </c>
+      <c r="C21" s="1">
+        <v>1.218183</v>
+      </c>
+      <c r="D21" s="1">
+        <v>1687.2726680000001</v>
+      </c>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1">
+        <v>553.4994814043755</v>
+      </c>
+      <c r="G21" s="1"/>
+      <c r="H21" s="1">
+        <v>6355.7575124384803</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" t="s">
+        <v>53</v>
+      </c>
+      <c r="C22" s="1">
+        <v>1687.2726680000001</v>
+      </c>
+      <c r="D22" s="1"/>
+      <c r="E22" s="1">
+        <v>546.41588891661229</v>
+      </c>
+      <c r="F22" s="1"/>
+      <c r="G22" s="1">
+        <v>7100.7972621620174</v>
+      </c>
+      <c r="H22" s="1"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="1">
+        <v>2336.210388476667</v>
+      </c>
+      <c r="D23" s="1">
+        <v>67.359874000000019</v>
+      </c>
+      <c r="E23" s="1">
+        <v>67.359874000000005</v>
+      </c>
+      <c r="F23" s="1">
+        <v>2336.210388476667</v>
+      </c>
+      <c r="G23" s="1"/>
+      <c r="H23" s="1"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C24" s="1">
+        <v>9118.2420918038915</v>
+      </c>
+      <c r="D24" s="1">
+        <v>9468.7607427136081</v>
+      </c>
+      <c r="E24" s="1">
+        <v>18553.952676552359</v>
+      </c>
+      <c r="F24" s="1">
+        <v>19845.866366514001</v>
+      </c>
+      <c r="G24" s="1">
+        <v>44310.750899859238</v>
+      </c>
+      <c r="H24" s="1">
+        <v>47023.988773570287</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>58</v>
+      </c>
+      <c r="C25" s="1">
+        <v>262376.75111480377</v>
+      </c>
+      <c r="D25" s="1">
+        <v>262376.75111480377</v>
+      </c>
+      <c r="E25" s="1">
+        <v>411778.16072249837</v>
+      </c>
+      <c r="F25" s="1">
+        <v>411778.16072249837</v>
+      </c>
+      <c r="G25" s="1">
+        <v>1624990.285015478</v>
+      </c>
+      <c r="H25" s="1">
+        <v>1624990.285015478</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>59</v>
+      </c>
+      <c r="C26" s="1"/>
+      <c r="D26" s="1"/>
+      <c r="E26" s="1"/>
+      <c r="F26" s="1"/>
+      <c r="G26" s="1">
+        <v>40692.357243687373</v>
+      </c>
+      <c r="H26" s="1"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1">
+        <v>-25100.98923128075</v>
+      </c>
+      <c r="F27" s="1">
+        <v>-25100.989231280721</v>
+      </c>
+      <c r="G27" s="1">
+        <v>147140.71535390709</v>
+      </c>
+      <c r="H27" s="1">
+        <v>147140.71535390709</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1">
+        <v>257299.2726750664</v>
+      </c>
+      <c r="G28" s="1">
+        <v>265583.73588885192</v>
+      </c>
+      <c r="H28" s="1"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1">
+        <v>154478.888047432</v>
+      </c>
+      <c r="F29" s="1">
+        <v>154478.888047432</v>
+      </c>
+      <c r="G29" s="1">
+        <v>1890574.0209043301</v>
+      </c>
+      <c r="H29" s="1">
+        <v>1890574.0209043301</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" t="s">
+        <v>59</v>
+      </c>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1">
+        <v>40692.357243687373</v>
+      </c>
+      <c r="H30" s="1"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>26</v>
+      </c>
+      <c r="B31" t="s">
+        <v>60</v>
+      </c>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1">
+        <v>-25100.989231280721</v>
+      </c>
+      <c r="F31" s="1">
+        <v>-25100.98923128075</v>
+      </c>
+      <c r="G31" s="1">
+        <v>147140.71535390709</v>
+      </c>
+      <c r="H31" s="1">
+        <v>147140.71535390709</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="1">
+        <v>62005.391748940048</v>
+      </c>
+      <c r="D32" s="1">
+        <v>62005.391748940048</v>
+      </c>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" s="1">
+        <v>86.331224277060215</v>
+      </c>
+      <c r="D33" s="1">
+        <v>-588.75960404294335</v>
+      </c>
+      <c r="E33" s="1">
+        <v>12747.614373</v>
+      </c>
+      <c r="F33" s="1">
+        <v>-16666.700353216482</v>
+      </c>
+      <c r="G33" s="1">
+        <v>9842.7329942164833</v>
+      </c>
+      <c r="H33" s="1">
+        <v>-8521.0363039999993</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="1">
+        <v>63134.524836636163</v>
+      </c>
+      <c r="D34" s="1">
+        <v>63134.515306242713</v>
+      </c>
+      <c r="E34" s="1">
+        <v>-60032.164387225363</v>
+      </c>
+      <c r="F34" s="1">
+        <v>-60032.164387225363</v>
+      </c>
+      <c r="G34" s="1">
+        <v>50492.474199902237</v>
+      </c>
+      <c r="H34" s="1">
+        <v>50492.474199901873</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>31</v>
+      </c>
+      <c r="B35" t="s">
+        <v>65</v>
+      </c>
+      <c r="C35" s="1">
+        <v>63134.515306242713</v>
+      </c>
+      <c r="D35" s="1">
+        <v>63134.524836636163</v>
+      </c>
+      <c r="E35" s="1">
+        <v>-60032.164387225363</v>
+      </c>
+      <c r="F35" s="1">
+        <v>-60032.164387225363</v>
+      </c>
+      <c r="G35" s="1">
+        <v>50492.474199901873</v>
+      </c>
+      <c r="H35" s="1">
+        <v>50492.474199902237</v>
       </c>
     </row>
     <row r="36">
@@ -4345,49 +5983,49 @@
       <c r="C36" s="1"/>
       <c r="D36" s="1"/>
       <c r="E36" s="1">
-        <v>200663.39336498949</v>
+        <v>264574.52162751998</v>
       </c>
       <c r="F36" s="1">
-        <v>200663.39336498949</v>
+        <v>264574.52162751998</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B37" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C37" s="1"/>
       <c r="D37" s="1"/>
       <c r="E37" s="1">
-        <v>1691.532447066628</v>
+        <v>272538.25067318691</v>
       </c>
       <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
+      <c r="G37" s="1">
+        <v>456.40441621169998</v>
+      </c>
+      <c r="H37" s="1">
+        <v>335741.85541967727</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C38" s="1"/>
       <c r="D38" s="1"/>
       <c r="E38" s="1">
-        <v>239376.743428952</v>
+        <v>1891.473003789004</v>
       </c>
       <c r="F38" s="1"/>
-      <c r="G38" s="1">
-        <v>402.67289956090139</v>
-      </c>
-      <c r="H38" s="1">
-        <v>298520.24294644757</v>
-      </c>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>